<commit_message>
improvements to TMS artefact removal, statistics, erserd analysis, eeg conversion
</commit_message>
<xml_diff>
--- a/template_files/template_parameters_analysis.xlsx
+++ b/template_files/template_parameters_analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0112736/Documents/MATLAB/net/template_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jessi\Desktop\net-master2025\template_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{308245B2-6869-624C-BD27-765D93C25F06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E9A63D1-8381-4009-9D07-AE9DDE66B072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10060" yWindow="760" windowWidth="20180" windowHeight="16100" activeTab="1" xr2:uid="{6EC9E106-9E35-B247-8D86-0F73FA459190}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{6EC9E106-9E35-B247-8D86-0F73FA459190}"/>
   </bookViews>
   <sheets>
     <sheet name="activity_analysis" sheetId="1" r:id="rId1"/>
@@ -247,9 +247,6 @@
     <t>all</t>
   </si>
   <si>
-    <t xml:space="preserve"> 'all', 'none' or list of dataset separated by spaces</t>
-  </si>
-  <si>
     <t>stats.demean</t>
   </si>
   <si>
@@ -329,6 +326,9 @@
   </si>
   <si>
     <t>template_triggers</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'all', 'none' or e.g [1 3] [7] [9 15]</t>
   </si>
 </sst>
 </file>
@@ -794,9 +794,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -834,7 +834,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -940,7 +940,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1082,7 +1082,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1091,7 +1091,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA96650F-26AA-EB46-99D2-C59E442E4347}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.5" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" style="2" bestFit="1" customWidth="1"/>
@@ -1099,7 +1099,7 @@
     <col min="4" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1110,7 +1110,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1132,18 +1132,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>10</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A6" s="12" t="s">
         <v>11</v>
       </c>
@@ -1165,7 +1165,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
         <v>13</v>
       </c>
@@ -1176,18 +1176,18 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
         <v>15</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C8" s="17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A9" s="18" t="s">
         <v>17</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A10" s="18" t="s">
         <v>18</v>
       </c>
@@ -1209,18 +1209,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A11" s="21" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C11" s="23" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A12" s="18" t="s">
         <v>20</v>
       </c>
@@ -1231,7 +1231,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A13" s="24" t="s">
         <v>21</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A14" s="24" t="s">
         <v>22</v>
       </c>
@@ -1253,12 +1253,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A15" s="27" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C15" s="29" t="s">
         <v>16</v>
@@ -1280,7 +1280,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B89B74C7-BC73-5F44-99BC-879A3B054F87}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.5" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41.1640625" style="2" customWidth="1"/>
@@ -1288,7 +1288,7 @@
     <col min="4" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -1299,7 +1299,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>24</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A3" s="12" t="s">
         <v>25</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A4" s="12" t="s">
         <v>26</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A5" s="12" t="s">
         <v>28</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A6" s="12" t="s">
         <v>30</v>
       </c>
@@ -1354,7 +1354,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
         <v>32</v>
       </c>
@@ -1365,7 +1365,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A8" s="12" t="s">
         <v>34</v>
       </c>
@@ -1376,7 +1376,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A9" s="12" t="s">
         <v>37</v>
       </c>
@@ -1387,7 +1387,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A10" s="12" t="s">
         <v>40</v>
       </c>
@@ -1398,16 +1398,16 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A12" s="18" t="s">
         <v>43</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A13" s="18" t="s">
         <v>44</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A14" s="24" t="s">
         <v>45</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A15" s="24" t="s">
         <v>46</v>
       </c>
@@ -1451,7 +1451,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A16" s="21" t="s">
         <v>47</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A17" s="21" t="s">
         <v>50</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A18" s="21" t="s">
         <v>53</v>
       </c>
@@ -1484,24 +1484,24 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A19" s="21" t="s">
         <v>55</v>
       </c>
       <c r="B19" s="35" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C19" s="23" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A20" s="36" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B20" s="37"/>
       <c r="C20" s="38" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1520,14 +1520,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A225D7CE-8777-D54B-A402-94CEC95943B4}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="25" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="25" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="69.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A2" s="40" t="s">
         <v>56</v>
       </c>
@@ -1546,10 +1546,10 @@
         <v>57</v>
       </c>
       <c r="C2" s="41" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A3" s="40" t="s">
         <v>58</v>
       </c>
@@ -1557,106 +1557,106 @@
         <v>59</v>
       </c>
       <c r="C3" s="40" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="42" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A4" s="42" t="s">
+      <c r="B4" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="42" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="C5" s="42" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="42" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="42" t="s">
         <v>69</v>
       </c>
-      <c r="C4" s="42" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A5" s="42" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" s="42" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="42" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A6" s="42" t="s">
-        <v>66</v>
-      </c>
-      <c r="B6" s="42" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" s="42" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A7" s="42" t="s">
+    </row>
+    <row r="8" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="42" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="42" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="42" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="42" t="s">
+      <c r="C8" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="42" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="42" t="s">
+    </row>
+    <row r="9" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="40" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="19" x14ac:dyDescent="0.2">
-      <c r="A9" s="40" t="s">
+      <c r="B9" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="B9" s="40" t="s">
+      <c r="C9" s="43" t="s">
         <v>74</v>
       </c>
-      <c r="C9" s="43" t="s">
+    </row>
+    <row r="10" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="40" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A10" s="40" t="s">
-        <v>76</v>
       </c>
       <c r="B10" s="40">
         <v>5000</v>
       </c>
       <c r="C10" s="40" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="40" t="s">
         <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="19" x14ac:dyDescent="0.2">
-      <c r="A11" s="40" t="s">
-        <v>78</v>
       </c>
       <c r="B11" s="40">
         <v>0.05</v>
       </c>
       <c r="C11" s="43" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="44" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A12" s="44" t="s">
+      <c r="B12" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="44" t="s">
         <v>80</v>
-      </c>
-      <c r="B12" s="44" t="s">
-        <v>69</v>
-      </c>
-      <c r="C12" s="44" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>